<commit_message>
Ajout d'une capture d'ecran par detail dans le classeur de suivi
- Feuille "Suivi general" : colonne Capture, image du rendu galerie
  (controle/galerie/folio_NN.png) pour chaque ligne rattachee a un folio
  unique (44/48 lignes ; les 4 transverses T2-T5 n'ont pas de folio unique
  donc pas d'image, T1 illustre par la page de garde)
- Feuille "Points bloquants" : capture pour les points 3/4/5 (folios 38,
  45, 27 respectivement) ; points 1/2 transverses sans capture
- Images redimensionnees a 300px de large (proportions conservees),
  ancrage OneCellAnchor verifie dans le XML OOXML genere
- Verification : images extraites du zip xlsx et relues individuellement
  (contenu correct, page de garde lisible) ; LibreOffice headless de cet
  environnement echoue a charger meme le fichier modele original (limite
  d'environnement, pas du fichier genere)

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017VbAyN4ZCNL12BkNusqYAa
</commit_message>
<xml_diff>
--- a/docs/Carnet_etancheite_suivi_avancement_v02.xlsx
+++ b/docs/Carnet_etancheite_suivi_avancement_v02.xlsx
@@ -181,7 +181,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -199,6 +199,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -223,6 +224,7 @@
     <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -312,6 +314,1191 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="2019300"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>11</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1714500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>12</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1714500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>13</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>15</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>16</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="9" name="Image 9" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="10" name="Image 10" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>18</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="11" name="Image 11" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="12" name="Image 12" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>20</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="13" name="Image 13" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId13"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="14" name="Image 14" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId14"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>22</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="15" name="Image 15" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId15"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>23</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="16" name="Image 16" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId16"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>24</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="17" name="Image 17" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId17"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="18" name="Image 18" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId18"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>26</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="19" name="Image 19" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId19"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>27</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1714500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="20" name="Image 20" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId20"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>28</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1714500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="21" name="Image 21" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId21"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>29</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="22" name="Image 22" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId22"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>30</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="23" name="Image 23" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId23"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>31</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1714500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="24" name="Image 24" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId24"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>32</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="25" name="Image 25" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId25"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>33</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1714500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="26" name="Image 26" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId26"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>34</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="27" name="Image 27" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId27"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>35</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="28" name="Image 28" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId28"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>36</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="29" name="Image 29" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId29"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>37</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="30" name="Image 30" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId30"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>38</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="31" name="Image 31" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId31"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>39</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="32" name="Image 32" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId32"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>40</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="33" name="Image 33" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId33"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>41</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="34" name="Image 34" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId34"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>42</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="35" name="Image 35" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId35"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>43</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="36" name="Image 36" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId36"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>44</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="37" name="Image 37" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId37"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>45</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="38" name="Image 38" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId38"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>46</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="39" name="Image 39" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId39"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>47</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="40" name="Image 40" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId40"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>48</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="41" name="Image 41" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId41"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>49</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="42" name="Image 42" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId42"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>50</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="43" name="Image 43" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId43"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>51</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="44" name="Image 44" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId44"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>6</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>8</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2857500" cy="1543050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -603,7 +1790,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H62"/>
+  <dimension ref="A1:I62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -614,6 +1801,7 @@
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -671,8 +1859,13 @@
           <t>Commentaire</t>
         </is>
       </c>
-    </row>
-    <row r="5">
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Capture</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="165.36" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>T1</t>
@@ -705,6 +1898,7 @@
           <t>Valeurs de contrôle C1 p.81 déjà rassemblées dans le mail</t>
         </is>
       </c>
+      <c r="I5" s="7" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -728,7 +1922,7 @@
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr"/>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="F6" s="8" t="inlineStr">
         <is>
           <t>Fait partiellement</t>
         </is>
@@ -743,6 +1937,7 @@
           <t>Épaisseur écran sup. = point bloquant n°2</t>
         </is>
       </c>
+      <c r="I6" s="7" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -770,7 +1965,7 @@
           <t>05/07/2026</t>
         </is>
       </c>
-      <c r="F7" s="8" t="inlineStr">
+      <c r="F7" s="9" t="inlineStr">
         <is>
           <t>Fait</t>
         </is>
@@ -781,6 +1976,7 @@
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr"/>
+      <c r="I7" s="7" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -808,7 +2004,7 @@
           <t>05/07/2026</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="F8" s="9" t="inlineStr">
         <is>
           <t>Fait</t>
         </is>
@@ -819,6 +2015,7 @@
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr"/>
+      <c r="I8" s="7" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -846,7 +2043,7 @@
           <t>06/07/2026</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="F9" s="8" t="inlineStr">
         <is>
           <t>Fait partiellement</t>
         </is>
@@ -861,8 +2058,9 @@
           <t>Prescription générale à porter au futur folio 00</t>
         </is>
       </c>
-    </row>
-    <row r="10">
+      <c r="I9" s="7" t="n"/>
+    </row>
+    <row r="10" ht="126.36" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>P1</t>
@@ -888,7 +2086,7 @@
           <t>06/07/2026</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
+      <c r="F10" s="9" t="inlineStr">
         <is>
           <t>Fait</t>
         </is>
@@ -899,8 +2097,9 @@
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr"/>
-    </row>
-    <row r="11">
+      <c r="I10" s="7" t="n"/>
+    </row>
+    <row r="11" ht="126.36" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>P2</t>
@@ -926,7 +2125,7 @@
           <t>05/07/2026</t>
         </is>
       </c>
-      <c r="F11" s="8" t="inlineStr">
+      <c r="F11" s="9" t="inlineStr">
         <is>
           <t>Fait</t>
         </is>
@@ -937,8 +2136,9 @@
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr"/>
-    </row>
-    <row r="12">
+      <c r="I11" s="7" t="n"/>
+    </row>
+    <row r="12" ht="140.4" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>P4/P20</t>
@@ -956,7 +2156,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr"/>
       <c r="E12" s="4" t="inlineStr"/>
-      <c r="F12" s="9" t="inlineStr">
+      <c r="F12" s="10" t="inlineStr">
         <is>
           <t>Question</t>
         </is>
@@ -971,8 +2171,9 @@
           <t>Le mail ne tranche pas la cible : époxy ou polymérique ?</t>
         </is>
       </c>
-    </row>
-    <row r="13">
+      <c r="I12" s="7" t="n"/>
+    </row>
+    <row r="13" ht="140.4" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
           <t>P8</t>
@@ -998,7 +2199,7 @@
           <t>05/07/2026</t>
         </is>
       </c>
-      <c r="F13" s="8" t="inlineStr">
+      <c r="F13" s="9" t="inlineStr">
         <is>
           <t>Fait</t>
         </is>
@@ -1009,8 +2210,9 @@
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr"/>
-    </row>
-    <row r="14">
+      <c r="I13" s="7" t="n"/>
+    </row>
+    <row r="14" ht="126.36" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>P9</t>
@@ -1036,7 +2238,7 @@
           <t>05/07/2026</t>
         </is>
       </c>
-      <c r="F14" s="8" t="inlineStr">
+      <c r="F14" s="9" t="inlineStr">
         <is>
           <t>Fait</t>
         </is>
@@ -1047,8 +2249,9 @@
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr"/>
-    </row>
-    <row r="15">
+      <c r="I14" s="7" t="n"/>
+    </row>
+    <row r="15" ht="126.36" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
           <t>P10</t>
@@ -1081,8 +2284,9 @@
           <t>Folio à créer n°2 de la liste</t>
         </is>
       </c>
-    </row>
-    <row r="16">
+      <c r="I15" s="7" t="n"/>
+    </row>
+    <row r="16" ht="126.36" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>P11,16-19</t>
@@ -1100,7 +2304,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr"/>
       <c r="E16" s="4" t="inlineStr"/>
-      <c r="F16" s="9" t="inlineStr">
+      <c r="F16" s="10" t="inlineStr">
         <is>
           <t>Question</t>
         </is>
@@ -1115,8 +2319,9 @@
           <t>Pas d'anomalie objective au rendu ; critère de cible à préciser</t>
         </is>
       </c>
-    </row>
-    <row r="17">
+      <c r="I16" s="7" t="n"/>
+    </row>
+    <row r="17" ht="126.36" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
           <t>P12-14 a</t>
@@ -1142,7 +2347,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F17" s="8" t="inlineStr">
+      <c r="F17" s="9" t="inlineStr">
         <is>
           <t>Déjà conforme</t>
         </is>
@@ -1153,8 +2358,9 @@
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr"/>
-    </row>
-    <row r="18">
+      <c r="I17" s="7" t="n"/>
+    </row>
+    <row r="18" ht="126.36" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
           <t>P12-14 b</t>
@@ -1172,7 +2378,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr"/>
       <c r="E18" s="4" t="inlineStr"/>
-      <c r="F18" s="9" t="inlineStr">
+      <c r="F18" s="10" t="inlineStr">
         <is>
           <t>Question</t>
         </is>
@@ -1187,8 +2393,9 @@
           <t>Ambiguïté signalée par le mail lui-même</t>
         </is>
       </c>
-    </row>
-    <row r="19">
+      <c r="I18" s="7" t="n"/>
+    </row>
+    <row r="19" ht="126.36" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
           <t>P15</t>
@@ -1214,7 +2421,7 @@
           <t>06/07/2026</t>
         </is>
       </c>
-      <c r="F19" s="8" t="inlineStr">
+      <c r="F19" s="9" t="inlineStr">
         <is>
           <t>Fait</t>
         </is>
@@ -1225,8 +2432,9 @@
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr"/>
-    </row>
-    <row r="20">
+      <c r="I19" s="7" t="n"/>
+    </row>
+    <row r="20" ht="126.36" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
           <t>P20</t>
@@ -1252,7 +2460,7 @@
           <t>05/07/2026</t>
         </is>
       </c>
-      <c r="F20" s="8" t="inlineStr">
+      <c r="F20" s="9" t="inlineStr">
         <is>
           <t>Fait</t>
         </is>
@@ -1263,8 +2471,9 @@
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr"/>
-    </row>
-    <row r="21">
+      <c r="I20" s="7" t="n"/>
+    </row>
+    <row r="21" ht="126.36" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
           <t>P21</t>
@@ -1290,7 +2499,7 @@
           <t>06/07/2026</t>
         </is>
       </c>
-      <c r="F21" s="7" t="inlineStr">
+      <c r="F21" s="8" t="inlineStr">
         <is>
           <t>Fait partiellement</t>
         </is>
@@ -1305,8 +2514,9 @@
           <t>Vérification des cotes 22-25 vs principe : revue Alexandre</t>
         </is>
       </c>
-    </row>
-    <row r="22">
+      <c r="I21" s="7" t="n"/>
+    </row>
+    <row r="22" ht="126.36" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>P22/23</t>
@@ -1332,7 +2542,7 @@
           <t>05/07/2026</t>
         </is>
       </c>
-      <c r="F22" s="8" t="inlineStr">
+      <c r="F22" s="9" t="inlineStr">
         <is>
           <t>Fait</t>
         </is>
@@ -1343,8 +2553,9 @@
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr"/>
-    </row>
-    <row r="23">
+      <c r="I22" s="7" t="n"/>
+    </row>
+    <row r="23" ht="126.36" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
           <t>P24</t>
@@ -1370,7 +2581,7 @@
           <t>05/07/2026</t>
         </is>
       </c>
-      <c r="F23" s="8" t="inlineStr">
+      <c r="F23" s="9" t="inlineStr">
         <is>
           <t>Fait</t>
         </is>
@@ -1381,8 +2592,9 @@
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr"/>
-    </row>
-    <row r="24">
+      <c r="I23" s="7" t="n"/>
+    </row>
+    <row r="24" ht="126.36" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
           <t>P25</t>
@@ -1408,7 +2620,7 @@
           <t>05/07/2026</t>
         </is>
       </c>
-      <c r="F24" s="8" t="inlineStr">
+      <c r="F24" s="9" t="inlineStr">
         <is>
           <t>Fait</t>
         </is>
@@ -1419,8 +2631,9 @@
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr"/>
-    </row>
-    <row r="25">
+      <c r="I24" s="7" t="n"/>
+    </row>
+    <row r="25" ht="126.36" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
           <t>P27 a</t>
@@ -1438,7 +2651,7 @@
       </c>
       <c r="D25" s="4" t="inlineStr"/>
       <c r="E25" s="4" t="inlineStr"/>
-      <c r="F25" s="10" t="inlineStr">
+      <c r="F25" s="11" t="inlineStr">
         <is>
           <t>Bloqué</t>
         </is>
@@ -1453,8 +2666,9 @@
           <t>Point bloquant n°5 — règle interne ou à sourcer</t>
         </is>
       </c>
-    </row>
-    <row r="26">
+      <c r="I25" s="7" t="n"/>
+    </row>
+    <row r="26" ht="126.36" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
           <t>P27 b</t>
@@ -1480,7 +2694,7 @@
           <t>05/07/2026</t>
         </is>
       </c>
-      <c r="F26" s="8" t="inlineStr">
+      <c r="F26" s="9" t="inlineStr">
         <is>
           <t>Fait</t>
         </is>
@@ -1491,8 +2705,9 @@
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr"/>
-    </row>
-    <row r="27">
+      <c r="I26" s="7" t="n"/>
+    </row>
+    <row r="27" ht="126.36" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
         <is>
           <t>P29</t>
@@ -1518,7 +2733,7 @@
           <t>05/07/2026</t>
         </is>
       </c>
-      <c r="F27" s="8" t="inlineStr">
+      <c r="F27" s="9" t="inlineStr">
         <is>
           <t>Fait</t>
         </is>
@@ -1529,8 +2744,9 @@
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr"/>
-    </row>
-    <row r="28">
+      <c r="I27" s="7" t="n"/>
+    </row>
+    <row r="28" ht="140.4" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
           <t>P30/32</t>
@@ -1556,7 +2772,7 @@
           <t>06/07/2026</t>
         </is>
       </c>
-      <c r="F28" s="7" t="inlineStr">
+      <c r="F28" s="8" t="inlineStr">
         <is>
           <t>Fait partiellement</t>
         </is>
@@ -1567,8 +2783,9 @@
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr"/>
-    </row>
-    <row r="29">
+      <c r="I28" s="7" t="n"/>
+    </row>
+    <row r="29" ht="140.4" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
           <t>P31/33</t>
@@ -1594,7 +2811,7 @@
           <t>05/07/2026</t>
         </is>
       </c>
-      <c r="F29" s="8" t="inlineStr">
+      <c r="F29" s="9" t="inlineStr">
         <is>
           <t>Fait</t>
         </is>
@@ -1605,8 +2822,9 @@
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
-    </row>
-    <row r="30">
+      <c r="I29" s="7" t="n"/>
+    </row>
+    <row r="30" ht="126.36" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
           <t>P34 a</t>
@@ -1632,7 +2850,7 @@
           <t>05/07/2026</t>
         </is>
       </c>
-      <c r="F30" s="8" t="inlineStr">
+      <c r="F30" s="9" t="inlineStr">
         <is>
           <t>Fait</t>
         </is>
@@ -1643,8 +2861,9 @@
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
-    </row>
-    <row r="31">
+      <c r="I30" s="7" t="n"/>
+    </row>
+    <row r="31" ht="126.36" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
         <is>
           <t>P34/36 b</t>
@@ -1670,7 +2889,7 @@
           <t>05/07/2026 / 06/07/2026</t>
         </is>
       </c>
-      <c r="F31" s="8" t="inlineStr">
+      <c r="F31" s="9" t="inlineStr">
         <is>
           <t>Fait</t>
         </is>
@@ -1681,8 +2900,9 @@
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
-    </row>
-    <row r="32">
+      <c r="I31" s="7" t="n"/>
+    </row>
+    <row r="32" ht="140.4" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
         <is>
           <t>P37</t>
@@ -1708,7 +2928,7 @@
           <t>05/07/2026</t>
         </is>
       </c>
-      <c r="F32" s="8" t="inlineStr">
+      <c r="F32" s="9" t="inlineStr">
         <is>
           <t>Fait</t>
         </is>
@@ -1719,8 +2939,9 @@
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
-    </row>
-    <row r="33">
+      <c r="I32" s="7" t="n"/>
+    </row>
+    <row r="33" ht="126.36" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
         <is>
           <t>P38</t>
@@ -1738,7 +2959,7 @@
       </c>
       <c r="D33" s="4" t="inlineStr"/>
       <c r="E33" s="4" t="inlineStr"/>
-      <c r="F33" s="10" t="inlineStr">
+      <c r="F33" s="11" t="inlineStr">
         <is>
           <t>Bloqué</t>
         </is>
@@ -1753,8 +2974,9 @@
           <t>Point bloquant n°3</t>
         </is>
       </c>
-    </row>
-    <row r="34">
+      <c r="I33" s="7" t="n"/>
+    </row>
+    <row r="34" ht="140.4" customHeight="1">
       <c r="A34" s="4" t="inlineStr">
         <is>
           <t>P39</t>
@@ -1780,7 +3002,7 @@
           <t>05/07/2026</t>
         </is>
       </c>
-      <c r="F34" s="8" t="inlineStr">
+      <c r="F34" s="9" t="inlineStr">
         <is>
           <t>Fait</t>
         </is>
@@ -1791,8 +3013,9 @@
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
-    </row>
-    <row r="35">
+      <c r="I34" s="7" t="n"/>
+    </row>
+    <row r="35" ht="126.36" customHeight="1">
       <c r="A35" s="4" t="inlineStr">
         <is>
           <t>P41</t>
@@ -1818,7 +3041,7 @@
           <t>05/07/2026</t>
         </is>
       </c>
-      <c r="F35" s="8" t="inlineStr">
+      <c r="F35" s="9" t="inlineStr">
         <is>
           <t>Fait</t>
         </is>
@@ -1829,8 +3052,9 @@
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
-    </row>
-    <row r="36">
+      <c r="I35" s="7" t="n"/>
+    </row>
+    <row r="36" ht="126.36" customHeight="1">
       <c r="A36" s="4" t="inlineStr">
         <is>
           <t>P44</t>
@@ -1856,7 +3080,7 @@
           <t>05/07/2026</t>
         </is>
       </c>
-      <c r="F36" s="8" t="inlineStr">
+      <c r="F36" s="9" t="inlineStr">
         <is>
           <t>Fait</t>
         </is>
@@ -1867,8 +3091,9 @@
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
-    </row>
-    <row r="37">
+      <c r="I36" s="7" t="n"/>
+    </row>
+    <row r="37" ht="126.36" customHeight="1">
       <c r="A37" s="4" t="inlineStr">
         <is>
           <t>P45 a</t>
@@ -1886,7 +3111,7 @@
       </c>
       <c r="D37" s="4" t="inlineStr"/>
       <c r="E37" s="4" t="inlineStr"/>
-      <c r="F37" s="10" t="inlineStr">
+      <c r="F37" s="11" t="inlineStr">
         <is>
           <t>Bloqué</t>
         </is>
@@ -1901,8 +3126,9 @@
           <t>Point bloquant n°4</t>
         </is>
       </c>
-    </row>
-    <row r="38">
+      <c r="I37" s="7" t="n"/>
+    </row>
+    <row r="38" ht="126.36" customHeight="1">
       <c r="A38" s="4" t="inlineStr">
         <is>
           <t>P45 b</t>
@@ -1928,7 +3154,7 @@
           <t>05/07/2026</t>
         </is>
       </c>
-      <c r="F38" s="8" t="inlineStr">
+      <c r="F38" s="9" t="inlineStr">
         <is>
           <t>Fait</t>
         </is>
@@ -1943,8 +3169,9 @@
           <t>Même texte au folio 63 (#13E13) non modifié : voir question</t>
         </is>
       </c>
-    </row>
-    <row r="39">
+      <c r="I38" s="7" t="n"/>
+    </row>
+    <row r="39" ht="126.36" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
         <is>
           <t>P47</t>
@@ -1970,7 +3197,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F39" s="9" t="inlineStr">
+      <c r="F39" s="10" t="inlineStr">
         <is>
           <t>Question</t>
         </is>
@@ -1985,8 +3212,9 @@
           <t>Généraliser 5-&gt;6cm partout ? voir question dédiée</t>
         </is>
       </c>
-    </row>
-    <row r="40">
+      <c r="I39" s="7" t="n"/>
+    </row>
+    <row r="40" ht="126.36" customHeight="1">
       <c r="A40" s="4" t="inlineStr">
         <is>
           <t>P48</t>
@@ -2004,7 +3232,7 @@
       </c>
       <c r="D40" s="4" t="inlineStr"/>
       <c r="E40" s="4" t="inlineStr"/>
-      <c r="F40" s="9" t="inlineStr">
+      <c r="F40" s="10" t="inlineStr">
         <is>
           <t>Question</t>
         </is>
@@ -2019,8 +3247,9 @@
           <t>Pas d'anomalie objective au rendu ; régression Lot2 corrigée au Lot4</t>
         </is>
       </c>
-    </row>
-    <row r="41">
+      <c r="I40" s="7" t="n"/>
+    </row>
+    <row r="41" ht="126.36" customHeight="1">
       <c r="A41" s="4" t="inlineStr">
         <is>
           <t>P49</t>
@@ -2046,7 +3275,7 @@
           <t>05/07/2026</t>
         </is>
       </c>
-      <c r="F41" s="8" t="inlineStr">
+      <c r="F41" s="9" t="inlineStr">
         <is>
           <t>Fait</t>
         </is>
@@ -2057,8 +3286,9 @@
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr"/>
-    </row>
-    <row r="42">
+      <c r="I41" s="7" t="n"/>
+    </row>
+    <row r="42" ht="126.36" customHeight="1">
       <c r="A42" s="4" t="inlineStr">
         <is>
           <t>P50</t>
@@ -2076,7 +3306,7 @@
       </c>
       <c r="D42" s="4" t="inlineStr"/>
       <c r="E42" s="4" t="inlineStr"/>
-      <c r="F42" s="11" t="inlineStr">
+      <c r="F42" s="12" t="inlineStr">
         <is>
           <t>À faire (dessin)</t>
         </is>
@@ -2091,8 +3321,9 @@
           <t>Nécessite entités graphiques, lot dédié</t>
         </is>
       </c>
-    </row>
-    <row r="43">
+      <c r="I42" s="7" t="n"/>
+    </row>
+    <row r="43" ht="126.36" customHeight="1">
       <c r="A43" s="4" t="inlineStr">
         <is>
           <t>P51</t>
@@ -2118,7 +3349,7 @@
           <t>05/07/2026</t>
         </is>
       </c>
-      <c r="F43" s="8" t="inlineStr">
+      <c r="F43" s="9" t="inlineStr">
         <is>
           <t>Fait</t>
         </is>
@@ -2129,8 +3360,9 @@
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr"/>
-    </row>
-    <row r="44">
+      <c r="I43" s="7" t="n"/>
+    </row>
+    <row r="44" ht="126.36" customHeight="1">
       <c r="A44" s="4" t="inlineStr">
         <is>
           <t>P52-54 a</t>
@@ -2156,7 +3388,7 @@
           <t>05/07/2026</t>
         </is>
       </c>
-      <c r="F44" s="8" t="inlineStr">
+      <c r="F44" s="9" t="inlineStr">
         <is>
           <t>Fait</t>
         </is>
@@ -2167,8 +3399,9 @@
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr"/>
-    </row>
-    <row r="45">
+      <c r="I44" s="7" t="n"/>
+    </row>
+    <row r="45" ht="126.36" customHeight="1">
       <c r="A45" s="4" t="inlineStr">
         <is>
           <t>P52-54 b</t>
@@ -2201,8 +3434,9 @@
           <t>Cite le Cahier 2 -&gt; dépend du point bloquant n°1</t>
         </is>
       </c>
-    </row>
-    <row r="46">
+      <c r="I45" s="7" t="n"/>
+    </row>
+    <row r="46" ht="126.36" customHeight="1">
       <c r="A46" s="4" t="inlineStr">
         <is>
           <t>P55/57/59</t>
@@ -2228,7 +3462,7 @@
           <t>05/07/2026</t>
         </is>
       </c>
-      <c r="F46" s="8" t="inlineStr">
+      <c r="F46" s="9" t="inlineStr">
         <is>
           <t>Fait</t>
         </is>
@@ -2239,8 +3473,9 @@
         </is>
       </c>
       <c r="H46" s="4" t="inlineStr"/>
-    </row>
-    <row r="47">
+      <c r="I46" s="7" t="n"/>
+    </row>
+    <row r="47" ht="126.36" customHeight="1">
       <c r="A47" s="4" t="inlineStr">
         <is>
           <t>P56-60</t>
@@ -2266,7 +3501,7 @@
           <t>05/07/2026</t>
         </is>
       </c>
-      <c r="F47" s="8" t="inlineStr">
+      <c r="F47" s="9" t="inlineStr">
         <is>
           <t>Fait</t>
         </is>
@@ -2277,8 +3512,9 @@
         </is>
       </c>
       <c r="H47" s="4" t="inlineStr"/>
-    </row>
-    <row r="48">
+      <c r="I47" s="7" t="n"/>
+    </row>
+    <row r="48" ht="126.36" customHeight="1">
       <c r="A48" s="4" t="inlineStr">
         <is>
           <t>P61 a</t>
@@ -2304,7 +3540,7 @@
           <t>05/07/2026</t>
         </is>
       </c>
-      <c r="F48" s="8" t="inlineStr">
+      <c r="F48" s="9" t="inlineStr">
         <is>
           <t>Fait</t>
         </is>
@@ -2315,8 +3551,9 @@
         </is>
       </c>
       <c r="H48" s="4" t="inlineStr"/>
-    </row>
-    <row r="49">
+      <c r="I48" s="7" t="n"/>
+    </row>
+    <row r="49" ht="126.36" customHeight="1">
       <c r="A49" s="4" t="inlineStr">
         <is>
           <t>P61 b</t>
@@ -2334,7 +3571,7 @@
       </c>
       <c r="D49" s="4" t="inlineStr"/>
       <c r="E49" s="4" t="inlineStr"/>
-      <c r="F49" s="9" t="inlineStr">
+      <c r="F49" s="10" t="inlineStr">
         <is>
           <t>Question</t>
         </is>
@@ -2349,8 +3586,9 @@
           <t>Vérification externe aux CMO des procédés prescrits</t>
         </is>
       </c>
-    </row>
-    <row r="50">
+      <c r="I49" s="7" t="n"/>
+    </row>
+    <row r="50" ht="126.36" customHeight="1">
       <c r="A50" s="4" t="inlineStr">
         <is>
           <t>P65 a</t>
@@ -2368,7 +3606,7 @@
       </c>
       <c r="D50" s="4" t="inlineStr"/>
       <c r="E50" s="4" t="inlineStr"/>
-      <c r="F50" s="9" t="inlineStr">
+      <c r="F50" s="10" t="inlineStr">
         <is>
           <t>Question</t>
         </is>
@@ -2383,8 +3621,9 @@
           <t>Valeur de remplacement à fournir</t>
         </is>
       </c>
-    </row>
-    <row r="51">
+      <c r="I50" s="7" t="n"/>
+    </row>
+    <row r="51" ht="126.36" customHeight="1">
       <c r="A51" s="4" t="inlineStr">
         <is>
           <t>P65 b</t>
@@ -2410,7 +3649,7 @@
           <t>05/07/2026</t>
         </is>
       </c>
-      <c r="F51" s="8" t="inlineStr">
+      <c r="F51" s="9" t="inlineStr">
         <is>
           <t>Fait</t>
         </is>
@@ -2421,8 +3660,9 @@
         </is>
       </c>
       <c r="H51" s="4" t="inlineStr"/>
-    </row>
-    <row r="52">
+      <c r="I51" s="7" t="n"/>
+    </row>
+    <row r="52" ht="126.36" customHeight="1">
       <c r="A52" s="4" t="inlineStr">
         <is>
           <t>P65 c</t>
@@ -2448,7 +3688,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F52" s="8" t="inlineStr">
+      <c r="F52" s="9" t="inlineStr">
         <is>
           <t>Déjà conforme</t>
         </is>
@@ -2459,100 +3699,102 @@
         </is>
       </c>
       <c r="H52" s="4" t="inlineStr"/>
+      <c r="I52" s="7" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="12" t="inlineStr">
+      <c r="A54" s="13" t="inlineStr">
         <is>
           <t>Synthèse :</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="13" t="inlineStr">
+      <c r="A55" s="14" t="inlineStr">
         <is>
           <t>Fait</t>
         </is>
       </c>
-      <c r="B55" s="14" t="n">
+      <c r="B55" s="15" t="n">
         <v>28</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="13" t="inlineStr">
+      <c r="A56" s="14" t="inlineStr">
         <is>
           <t>Fait partiellement</t>
         </is>
       </c>
-      <c r="B56" s="14" t="n">
+      <c r="B56" s="15" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="13" t="inlineStr">
+      <c r="A57" s="14" t="inlineStr">
         <is>
           <t>Déjà conforme</t>
         </is>
       </c>
-      <c r="B57" s="14" t="n">
+      <c r="B57" s="15" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="13" t="inlineStr">
+      <c r="A58" s="14" t="inlineStr">
         <is>
           <t>À faire (création)</t>
         </is>
       </c>
-      <c r="B58" s="14" t="n">
+      <c r="B58" s="15" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="13" t="inlineStr">
+      <c r="A59" s="14" t="inlineStr">
         <is>
           <t>À faire (dessin)</t>
         </is>
       </c>
-      <c r="B59" s="14" t="n">
+      <c r="B59" s="15" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="13" t="inlineStr">
+      <c r="A60" s="14" t="inlineStr">
         <is>
           <t>Bloqué</t>
         </is>
       </c>
-      <c r="B60" s="14" t="n">
+      <c r="B60" s="15" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="13" t="inlineStr">
+      <c r="A61" s="14" t="inlineStr">
         <is>
           <t>Question</t>
         </is>
       </c>
-      <c r="B61" s="14" t="n">
+      <c r="B61" s="15" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="14" t="inlineStr">
+      <c r="A62" s="15" t="inlineStr">
         <is>
           <t>Total items suivis</t>
         </is>
       </c>
-      <c r="B62" s="14" t="n">
+      <c r="B62" s="15" t="n">
         <v>48</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2562,7 +3804,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2570,6 +3812,7 @@
     <col width="70" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -2612,138 +3855,149 @@
           <t>Décision requise de</t>
         </is>
       </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Capture</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="n">
+      <c r="A5" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>Statut du Cahier 2 GT9</t>
         </is>
       </c>
-      <c r="C5" s="16" t="inlineStr">
+      <c r="C5" s="17" t="inlineStr">
         <is>
           <t>Cahier 2 (guide de choix, prépublication septembre 2025) : statut non confirmé. Ne pas citer comme référence contractuelle sans validation.</t>
         </is>
       </c>
-      <c r="D5" s="15" t="inlineStr">
+      <c r="D5" s="16" t="inlineStr">
         <is>
           <t>Folio 00 (à créer), P52-54 (tableau de choix)</t>
         </is>
       </c>
-      <c r="E5" s="15" t="inlineStr">
+      <c r="E5" s="16" t="inlineStr">
         <is>
           <t>Bertrand Verrière</t>
         </is>
       </c>
+      <c r="F5" s="18" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="n">
+      <c r="A6" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="17" t="inlineStr">
         <is>
           <t>Épaisseur écran supérieur DEG</t>
         </is>
       </c>
-      <c r="C6" s="16" t="inlineStr">
+      <c r="C6" s="17" t="inlineStr">
         <is>
           <t>Le GT9 C1F1 exige 19/10e mini, le carnet v01 indique 20/10e à plusieurs endroits. Confirmer la valeur cible pour la v02.</t>
         </is>
       </c>
-      <c r="D6" s="15" t="inlineStr">
+      <c r="D6" s="16" t="inlineStr">
         <is>
           <t>Légende complexe DEG (tous folios DEG)</t>
         </is>
       </c>
-      <c r="E6" s="15" t="inlineStr">
+      <c r="E6" s="16" t="inlineStr">
         <is>
           <t>Bertrand Verrière</t>
         </is>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="15" t="n">
+      <c r="F6" s="18" t="n"/>
+    </row>
+    <row r="7" ht="126.36" customHeight="1">
+      <c r="A7" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>Cotes d'engravure du folio 38</t>
         </is>
       </c>
-      <c r="C7" s="16" t="inlineStr">
+      <c r="C7" s="17" t="inlineStr">
         <is>
           <t>Valeurs actuelles (9/6/10/15 cm) à comparer aux CMO des procédés habituellement prescrits.</t>
         </is>
       </c>
-      <c r="D7" s="15" t="inlineStr">
+      <c r="D7" s="16" t="inlineStr">
         <is>
           <t>Folio 38</t>
         </is>
       </c>
-      <c r="E7" s="15" t="inlineStr">
+      <c r="E7" s="16" t="inlineStr">
         <is>
           <t>Bertrand Verrière</t>
         </is>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="15" t="n">
+      <c r="F7" s="18" t="n"/>
+    </row>
+    <row r="8" ht="126.36" customHeight="1">
+      <c r="A8" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="16" t="inlineStr">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>Raccord DEG/FPM du folio 45</t>
         </is>
       </c>
-      <c r="C8" s="16" t="inlineStr">
+      <c r="C8" s="17" t="inlineStr">
         <is>
           <t>Marqué «à définir» depuis la v01 (2022) : à trancher.</t>
         </is>
       </c>
-      <c r="D8" s="15" t="inlineStr">
+      <c r="D8" s="16" t="inlineStr">
         <is>
           <t>Folio 45</t>
         </is>
       </c>
-      <c r="E8" s="15" t="inlineStr">
+      <c r="E8" s="16" t="inlineStr">
         <is>
           <t>Bertrand Verrière</t>
         </is>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="15" t="n">
+      <c r="F8" s="18" t="n"/>
+    </row>
+    <row r="9" ht="126.36" customHeight="1">
+      <c r="A9" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="16" t="inlineStr">
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t>Seuil «hauteur d'eau &gt; 10 m» du folio 27</t>
         </is>
       </c>
-      <c r="C9" s="16" t="inlineStr">
+      <c r="C9" s="17" t="inlineStr">
         <is>
           <t>Règle interne à documenter, ou valeur à sourcer dans un référentiel.</t>
         </is>
       </c>
-      <c r="D9" s="15" t="inlineStr">
+      <c r="D9" s="16" t="inlineStr">
         <is>
           <t>Folio 27</t>
         </is>
       </c>
-      <c r="E9" s="15" t="inlineStr">
+      <c r="E9" s="16" t="inlineStr">
         <is>
           <t>Bertrand Verrière</t>
         </is>
       </c>
+      <c r="F9" s="18" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2799,160 +4053,160 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="17" t="n">
+      <c r="A5" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B5" s="20" t="inlineStr">
         <is>
           <t>Solin 3x3 cm</t>
         </is>
       </c>
-      <c r="C5" s="18" t="inlineStr">
+      <c r="C5" s="20" t="inlineStr">
         <is>
           <t>Mortier époxy (folio 4) ou polymérique (folio 20) : quelle cible unique ?</t>
         </is>
       </c>
-      <c r="D5" s="17" t="inlineStr">
+      <c r="D5" s="19" t="inlineStr">
         <is>
           <t>P4, P20</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="17" t="n">
+      <c r="A6" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="18" t="inlineStr">
+      <c r="B6" s="20" t="inlineStr">
         <is>
           <t>Béton de protection lourde 5 cm</t>
         </is>
       </c>
-      <c r="C6" s="18" t="inlineStr">
+      <c r="C6" s="20" t="inlineStr">
         <is>
           <t>Le folio 47 valide 6 cm pour les remontées d'édicules. Faut-il généraliser 5-&gt;6 cm partout (~12 occurrences, folios 15/33/34/40-43/46/48/51...) ou est-ce un autre élément (protection lourde horizontale) qui reste à 5 cm ?</t>
         </is>
       </c>
-      <c r="D6" s="17" t="inlineStr">
+      <c r="D6" s="19" t="inlineStr">
         <is>
           <t>P15, P33, P34, P40-43, P46, P48, P51...</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="17" t="n">
+      <c r="A7" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="18" t="inlineStr">
+      <c r="B7" s="20" t="inlineStr">
         <is>
           <t>Cote 0,50 m</t>
         </is>
       </c>
-      <c r="C7" s="18" t="inlineStr">
+      <c r="C7" s="20" t="inlineStr">
         <is>
           <t>Signification à confirmer avant de la légender.</t>
         </is>
       </c>
-      <c r="D7" s="17" t="inlineStr">
+      <c r="D7" s="19" t="inlineStr">
         <is>
           <t>P12-14</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="n">
+      <c r="A8" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="18" t="inlineStr">
+      <c r="B8" s="20" t="inlineStr">
         <is>
           <t>Engravure folio 65</t>
         </is>
       </c>
-      <c r="C8" s="18" t="inlineStr">
+      <c r="C8" s="20" t="inlineStr">
         <is>
           <t>«20x220 mm» signalée comme probablement erronée : valeur de remplacement ?</t>
         </is>
       </c>
-      <c r="D8" s="17" t="inlineStr">
+      <c r="D8" s="19" t="inlineStr">
         <is>
           <t>P65</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="n">
+      <c r="A9" s="19" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="18" t="inlineStr">
+      <c r="B9" s="20" t="inlineStr">
         <is>
           <t>Anti-racine folio 63</t>
         </is>
       </c>
-      <c r="C9" s="18" t="inlineStr">
+      <c r="C9" s="20" t="inlineStr">
         <is>
           <t>Même texte qu'au folio 45 (bicouche anti-racine) : appliquer la même condition «uniquement si végétalisation» ? Et le titre du folio 61 indique «D.E.G. - F.P.B» (F.P.B au lieu de F.P.M ailleurs) : coquille à confirmer.</t>
         </is>
       </c>
-      <c r="D9" s="17" t="inlineStr">
+      <c r="D9" s="19" t="inlineStr">
         <is>
           <t>P63, P61</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="n">
+      <c r="A10" s="19" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="18" t="inlineStr">
+      <c r="B10" s="20" t="inlineStr">
         <is>
           <t>Convention décimale</t>
         </is>
       </c>
-      <c r="C10" s="18" t="inlineStr">
+      <c r="C10" s="20" t="inlineStr">
         <is>
           <t>La source utilise le point partout (197 occurrences). La correction PDF «1,00m» impliquerait de basculer ~41 cotes en virgule. Bascule générale à trancher (charte Egis) avant toute modification massive.</t>
         </is>
       </c>
-      <c r="D10" s="17" t="inlineStr">
+      <c r="D10" s="19" t="inlineStr">
         <is>
           <t>Transverse</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="17" t="n">
+      <c r="A11" s="19" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="18" t="inlineStr">
+      <c r="B11" s="20" t="inlineStr">
         <is>
           <t>Casse/corps des libellés</t>
         </is>
       </c>
-      <c r="C11" s="18" t="inlineStr">
+      <c r="C11" s="20" t="inlineStr">
         <is>
           <t>Folios 11, 16-19 : casse hétérogène signalée par le mail, mais pas d'anomalie objective identifiée au rendu. Quel est le critère de cible ?</t>
         </is>
       </c>
-      <c r="D11" s="17" t="inlineStr">
+      <c r="D11" s="19" t="inlineStr">
         <is>
           <t>P11, P16-19</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="17" t="n">
+      <c r="A12" s="19" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="18" t="inlineStr">
+      <c r="B12" s="20" t="inlineStr">
         <is>
           <t>Casse/unites folio 48</t>
         </is>
       </c>
-      <c r="C12" s="18" t="inlineStr">
+      <c r="C12" s="20" t="inlineStr">
         <is>
           <t>Idem : pas d'anomalie objective au rendu (une régression du lot 2 sur le feuillard a été corrigée au lot 4). Cible d'harmonisation à préciser.</t>
         </is>
       </c>
-      <c r="D12" s="17" t="inlineStr">
+      <c r="D12" s="19" t="inlineStr">
         <is>
           <t>P48</t>
         </is>
@@ -3019,7 +4273,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="19" t="n">
+      <c r="A5" s="21" t="n">
         <v>1</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -3032,14 +4286,14 @@
           <t>F67-III, GT9.C1F1, GT9.C2 (sous réserve), GT9.R19F1, NF EN 13491/13256, AT CETU, ASQUAL soudeurs, réception support = point d'arrêt, valeurs de contrôle C1 p.81.</t>
         </is>
       </c>
-      <c r="D5" s="20" t="inlineStr">
+      <c r="D5" s="22" t="inlineStr">
         <is>
           <t>À faire (création)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="19" t="n">
+      <c r="A6" s="21" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -3052,14 +4306,14 @@
           <t>Bride/contre-bride ou tole colaminée — aujourd'hui traité par un simple solin (folio 10).</t>
         </is>
       </c>
-      <c r="D6" s="20" t="inlineStr">
+      <c r="D6" s="22" t="inlineStr">
         <is>
           <t>À faire (création)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="n">
+      <c r="A7" s="21" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -3072,14 +4326,14 @@
           <t>Géocomposite piédroit, barbacane, cunette raccordée, selon GT9.R19F1.</t>
         </is>
       </c>
-      <c r="D7" s="20" t="inlineStr">
+      <c r="D7" s="22" t="inlineStr">
         <is>
           <t>À faire (création)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="n">
+      <c r="A8" s="21" t="n">
         <v>4</v>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -3092,14 +4346,14 @@
           <t>Fourreaux, manchettes — hors bride/contre-bride.</t>
         </is>
       </c>
-      <c r="D8" s="20" t="inlineStr">
+      <c r="D8" s="22" t="inlineStr">
         <is>
           <t>À faire (création)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="n">
+      <c r="A9" s="21" t="n">
         <v>5</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -3112,14 +4366,14 @@
           <t>Par partie d'ouvrage et hauteur d'eau, inspiré du Cahier 2 §4.5 et §8.</t>
         </is>
       </c>
-      <c r="D9" s="21" t="inlineStr">
+      <c r="D9" s="23" t="inlineStr">
         <is>
           <t>Bloqué</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="n">
+      <c r="A10" s="21" t="n">
         <v>6</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -3132,7 +4386,7 @@
           <t>Détail non existant dans le carnet actuel.</t>
         </is>
       </c>
-      <c r="D10" s="20" t="inlineStr">
+      <c r="D10" s="22" t="inlineStr">
         <is>
           <t>À faire (création)</t>
         </is>

</xml_diff>

<commit_message>
normes N15+N16 FAIT: PDF final 72 pages + rapport justifie + Excel
- PDF couleur 72/72 pages (folio 00 + folios 66-70), controle visuel
  sur 15 pages, fix barres noires (masques MTEXT desactives au rendu),
  NOTA folio 46 repositionne dans la fenetre
- docs/rapport_maj_normes.md : 11 modifications tracees (quoi/folio/
  justification/norme), infos pour les 5 points bloques, divergences
  a arbitrer, manques documentaires (C6F1, R1F3)
- feuille Excel "MAJ normes 07-2026" (11 lignes) dans le classeur de
  suivi d'avancement
</commit_message>
<xml_diff>
--- a/docs/Carnet_etancheite_suivi_avancement_v02.xlsx
+++ b/docs/Carnet_etancheite_suivi_avancement_v02.xlsx
@@ -8,9 +8,10 @@
   </bookViews>
   <sheets>
     <sheet name="Suivi général" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Points bloquants" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Questions Alexandre" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Folios à créer" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="MAJ normes 07-2026" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Points bloquants" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Questions Alexandre" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Folios à créer" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -101,8 +102,13 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -154,8 +160,18 @@
         <fgColor rgb="00FFF9E0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002F5496"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -177,11 +193,25 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00999999"/>
+      </left>
+      <right style="thin">
+        <color rgb="00999999"/>
+      </right>
+      <top style="thin">
+        <color rgb="00999999"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00999999"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -239,6 +269,16 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -339,6 +379,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -364,6 +407,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -389,6 +435,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -414,6 +463,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -439,6 +491,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -464,6 +519,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -489,6 +547,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -514,6 +575,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -539,6 +603,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -564,6 +631,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -589,6 +659,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -614,6 +687,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -639,6 +715,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -664,6 +743,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -689,6 +771,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -714,6 +799,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -739,6 +827,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -764,6 +855,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -789,6 +883,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -814,6 +911,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -839,6 +939,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -864,6 +967,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -889,6 +995,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -914,6 +1023,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -939,6 +1051,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -964,6 +1079,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -989,6 +1107,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1014,6 +1135,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1039,6 +1163,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1064,6 +1191,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1089,6 +1219,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1114,6 +1247,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1139,6 +1275,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1164,6 +1303,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1189,6 +1331,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1214,6 +1359,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1239,6 +1387,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1264,6 +1415,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1289,6 +1443,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1314,6 +1471,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1339,6 +1499,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1364,6 +1527,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1389,6 +1555,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1414,6 +1583,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1444,6 +1616,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1469,6 +1644,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1494,6 +1672,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3804,6 +3985,290 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Folio(s)</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>Justification / Norme</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>Statut</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="25" t="inlineStr">
+        <is>
+          <t>15/33/34/40-43/46/48/51/61-63</t>
+        </is>
+      </c>
+      <c r="B2" s="25" t="inlineStr">
+        <is>
+          <t>Béton de protection lourde 5 cm -&gt; 6 cm (34 occ.)</t>
+        </is>
+      </c>
+      <c r="C2" s="25" t="inlineStr">
+        <is>
+          <t>GT9.C5F1 (prépub.) tableaux 1-3 ; cohérent P34/36 + P47 mail</t>
+        </is>
+      </c>
+      <c r="D2" s="26" t="inlineStr">
+        <is>
+          <t>FAIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="25" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B3" s="25" t="inlineStr">
+        <is>
+          <t>NOTA pipettes : &gt;=3/compartiment en boîtier poteau/refend</t>
+        </is>
+      </c>
+      <c r="C3" s="25" t="inlineStr">
+        <is>
+          <t>GT9.C10F1 §7.1 (publication)</t>
+        </is>
+      </c>
+      <c r="D3" s="26" t="inlineStr">
+        <is>
+          <t>FAIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="25" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="B4" s="25" t="inlineStr">
+        <is>
+          <t>NOTA surfaces maxi compartimentage 250/350 m²</t>
+        </is>
+      </c>
+      <c r="C4" s="25" t="inlineStr">
+        <is>
+          <t>F67-III art. 3.3.1</t>
+        </is>
+      </c>
+      <c r="D4" s="26" t="inlineStr">
+        <is>
+          <t>FAIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="25" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="B5" s="25" t="inlineStr">
+        <is>
+          <t>NOTA débit AFTES niveau 0 + retombée &gt;=20 cm</t>
+        </is>
+      </c>
+      <c r="C5" s="25" t="inlineStr">
+        <is>
+          <t>GT9.C10F1 §9</t>
+        </is>
+      </c>
+      <c r="D5" s="26" t="inlineStr">
+        <is>
+          <t>FAIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="25" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="B6" s="25" t="inlineStr">
+        <is>
+          <t>Grille anti-intrusion démontable + entretenabilité (graphique)</t>
+        </is>
+      </c>
+      <c r="C6" s="25" t="inlineStr">
+        <is>
+          <t>P50 mail ; GT9.C10F1 §9.3.1</t>
+        </is>
+      </c>
+      <c r="D6" s="26" t="inlineStr">
+        <is>
+          <t>FAIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="25" t="inlineStr">
+        <is>
+          <t>00 (créé)</t>
+        </is>
+      </c>
+      <c r="B7" s="25" t="inlineStr">
+        <is>
+          <t>Folio Références et généralités + contrôles C1 p.81</t>
+        </is>
+      </c>
+      <c r="C7" s="25" t="inlineStr">
+        <is>
+          <t>Mail Bertrand ; GT9.C1F1 p.81 ; F67-III §3.1-3.2</t>
+        </is>
+      </c>
+      <c r="D7" s="26" t="inlineStr">
+        <is>
+          <t>FAIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="25" t="inlineStr">
+        <is>
+          <t>66 (créé)</t>
+        </is>
+      </c>
+      <c r="B8" s="25" t="inlineStr">
+        <is>
+          <t>Arrêt DEG sur voussoir (tôle colaminée / bride-contre-bride)</t>
+        </is>
+      </c>
+      <c r="C8" s="25" t="inlineStr">
+        <is>
+          <t>GT9.C9F1 §6.5 (prépub.) ; F67-III §3.1.3.c</t>
+        </is>
+      </c>
+      <c r="D8" s="26" t="inlineStr">
+        <is>
+          <t>FAIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="25" t="inlineStr">
+        <is>
+          <t>67 (créé)</t>
+        </is>
+      </c>
+      <c r="B9" s="25" t="inlineStr">
+        <is>
+          <t>Détails drainage (nappe, cunette, collecteur)</t>
+        </is>
+      </c>
+      <c r="C9" s="25" t="inlineStr">
+        <is>
+          <t>GT9.R19F1 ; GT9.C10F1 §10.2</t>
+        </is>
+      </c>
+      <c r="D9" s="26" t="inlineStr">
+        <is>
+          <t>FAIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="25" t="inlineStr">
+        <is>
+          <t>68 (créé)</t>
+        </is>
+      </c>
+      <c r="B10" s="25" t="inlineStr">
+        <is>
+          <t>Traversées de réseaux courants (fourreau + hydrogonflant)</t>
+        </is>
+      </c>
+      <c r="C10" s="25" t="inlineStr">
+        <is>
+          <t>GT9.C10F1 §8 ; F67-III §3.1.7</t>
+        </is>
+      </c>
+      <c r="D10" s="26" t="inlineStr">
+        <is>
+          <t>FAIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="25" t="inlineStr">
+        <is>
+          <t>69 (créé)</t>
+        </is>
+      </c>
+      <c r="B11" s="25" t="inlineStr">
+        <is>
+          <t>Tableau de choix DEG/SEL-A/FPM — EN RÉSERVE</t>
+        </is>
+      </c>
+      <c r="C11" s="25" t="inlineStr">
+        <is>
+          <t>Dépend statut Cahier 2 = point BLOQUÉ n°1 (B. Verrière)</t>
+        </is>
+      </c>
+      <c r="D11" s="27" t="inlineStr">
+        <is>
+          <t>RÉSERVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="25" t="inlineStr">
+        <is>
+          <t>70 (créé)</t>
+        </is>
+      </c>
+      <c r="B12" s="25" t="inlineStr">
+        <is>
+          <t>Réparation/réinjection compartiment DEG (procédure)</t>
+        </is>
+      </c>
+      <c r="C12" s="25" t="inlineStr">
+        <is>
+          <t>GT9.R1F2 III.1.5.2.4</t>
+        </is>
+      </c>
+      <c r="D12" s="26" t="inlineStr">
+        <is>
+          <t>FAIT</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -4001,7 +4466,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4221,7 +4686,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>